<commit_message>
Support height-first module fields and upward independent turret geometry
</commit_message>
<xml_diff>
--- a/tools/data_source/game_data.xlsx
+++ b/tools/data_source/game_data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="R5b231fa8dc53463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="R0f865133d2f84446"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Rc99dbbe815c84a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="Re517e50d80604417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="R6554a5295d8e45b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="R9076678c438442b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="1" r:id="Rb7ac04d70fb4408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propulsion" sheetId="2" r:id="Rae807c20b4804282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapon" sheetId="3" r:id="Red2e815dd7544870"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defense" sheetId="4" r:id="R55e47db90030445d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Function" sheetId="5" r:id="Re2087cd3c8094683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="6" r:id="R70d3ffd9f8854fb0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,14 +286,14 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="7.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>标识</x:v>
       </x:c>
@@ -304,22 +304,20 @@
         <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>宽度</x:v>
+        <x:v>高X宽</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
-        <x:v>高度</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>能耗</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>贴图路径</x:v>
-      </x:c>
-      <x:c r="H1" s="10" t="str">
         <x:v>能量输出</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="H1" s="10"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
         <x:v>energy_smallreactor</x:v>
       </x:c>
@@ -329,22 +327,21 @@
       <x:c r="C2" s="11" t="str">
         <x:v>基础能量模块，为飞船提供持续能量。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
-        <x:v>1</x:v>
+      <x:c r="D2" s="11" t="str">
+        <x:v>1x1</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>res://data/assets/modules/energy_smallreactor.png</x:v>
       </x:c>
-      <x:c r="H2" s="11" t="n">
+      <x:c r="G2" s="11" t="n">
         <x:v>20</x:v>
       </x:c>
-    </x:row>
+      <x:c r="H2" s="11"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -357,14 +354,14 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="4.25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="4.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>标识</x:v>
       </x:c>
@@ -375,22 +372,20 @@
         <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>宽度</x:v>
+        <x:v>高X宽</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
-        <x:v>高度</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>能耗</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>贴图路径</x:v>
-      </x:c>
-      <x:c r="H1" s="10" t="str">
         <x:v>推力</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="H1" s="10"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
         <x:v>propulsion_smallengine</x:v>
       </x:c>
@@ -400,22 +395,21 @@
       <x:c r="C2" s="11" t="str">
         <x:v>基础动力模块，为飞船提供主要推进力。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
-        <x:v>1</x:v>
+      <x:c r="D2" s="11" t="str">
+        <x:v>1x1</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>res://data/assets/modules/propulsion_smallengine.png</x:v>
       </x:c>
-      <x:c r="H2" s="11" t="n">
+      <x:c r="G2" s="11" t="n">
         <x:v>20</x:v>
       </x:c>
-    </x:row>
+      <x:c r="H2" s="11"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -428,21 +422,24 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="7.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="7.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="15.25" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="9.75" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="41.880001068115234" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15.25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="9.75" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="41.880001068115234" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>标识</x:v>
       </x:c>
@@ -453,43 +450,52 @@
         <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>宽度</x:v>
+        <x:v>高X宽</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
-        <x:v>高度</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>能耗</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>贴图路径</x:v>
+        <x:v>火力</x:v>
       </x:c>
       <x:c r="H1" s="10" t="str">
-        <x:v>火力</x:v>
+        <x:v>攻击范围</x:v>
       </x:c>
       <x:c r="I1" s="10" t="str">
-        <x:v>攻击范围</x:v>
+        <x:v>射击间隔</x:v>
       </x:c>
       <x:c r="J1" s="10" t="str">
-        <x:v>射击间隔</x:v>
+        <x:v>炮塔转速（度/秒）</x:v>
       </x:c>
       <x:c r="K1" s="10" t="str">
-        <x:v>炮塔转速（度/秒）</x:v>
+        <x:v>弹速</x:v>
       </x:c>
       <x:c r="L1" s="10" t="str">
-        <x:v>弹速</x:v>
+        <x:v>开火角容差（度）</x:v>
       </x:c>
       <x:c r="M1" s="10" t="str">
-        <x:v>开火角容差（度）</x:v>
+        <x:v>射界（度）</x:v>
       </x:c>
       <x:c r="N1" s="10" t="str">
-        <x:v>射界（度）</x:v>
+        <x:v>炮塔贴图路径</x:v>
       </x:c>
       <x:c r="O1" s="10" t="str">
-        <x:v>炮塔贴图路径</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
+        <x:v>炮塔高X宽</x:v>
+      </x:c>
+      <x:c r="P1" s="10" t="str">
+        <x:v>炮塔轴点</x:v>
+      </x:c>
+      <x:c r="Q1" s="10" t="str">
+        <x:v>炮口</x:v>
+      </x:c>
+      <x:c r="R1" s="10" t="str">
+        <x:v>炮塔素材转角（度）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
         <x:v>weapon_cannon</x:v>
       </x:c>
@@ -499,43 +505,53 @@
       <x:c r="C2" s="11" t="str">
         <x:v>基础武器模块，提供稳定的常规火力。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
-        <x:v>1</x:v>
+      <x:c r="D2" s="11" t="str">
+        <x:v>1x1</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>res://data/assets/modules/weapon_cannon_base.png</x:v>
       </x:c>
+      <x:c r="G2" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="H2" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="I2" s="11" t="n">
-        <x:v>500</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="J2" s="11" t="n">
-        <x:v>0.5</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="K2" s="11" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="L2" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M2" s="11" t="n">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="L2" s="11" t="n">
-        <x:v>700</x:v>
-      </x:c>
-      <x:c r="M2" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="N2" s="11" t="n">
-        <x:v>180</x:v>
+      <x:c r="N2" s="11" t="str">
+        <x:v>res://data/assets/modules/weapon_cannon_turret.png</x:v>
       </x:c>
       <x:c r="O2" s="11" t="str">
-        <x:v>res://data/assets/modules/weapon_cannon_turret.png</x:v>
-      </x:c>
-    </x:row>
+        <x:v>2x1</x:v>
+      </x:c>
+      <x:c r="P2" s="11" t="str">
+        <x:v>0.5,0.25</x:v>
+      </x:c>
+      <x:c r="Q2" s="11" t="str">
+        <x:v>0.5,0.98</x:v>
+      </x:c>
+      <x:c r="R2" s="11" t="n">
+        <x:v>-90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -548,15 +564,15 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="6" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4.25" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="4.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>标识</x:v>
       </x:c>
@@ -567,25 +583,23 @@
         <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>宽度</x:v>
+        <x:v>高X宽</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
-        <x:v>高度</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>能耗</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>贴图路径</x:v>
+        <x:v>生命值</x:v>
       </x:c>
       <x:c r="H1" s="10" t="str">
-        <x:v>生命值</x:v>
-      </x:c>
-      <x:c r="I1" s="10" t="str">
         <x:v>防护</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="I1" s="10"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
         <x:v>defense_lightarmor</x:v>
       </x:c>
@@ -595,25 +609,24 @@
       <x:c r="C2" s="11" t="str">
         <x:v>基础防护模块，为飞船提供结构防护。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
+      <x:c r="D2" s="11" t="str">
+        <x:v>1x1</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>res://data/assets/modules/defense_lightarmor.png</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H2" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E2" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G2" s="11" t="str">
-        <x:v>res://data/assets/modules/defense_lightarmor.png</x:v>
-      </x:c>
-      <x:c r="H2" s="11" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="I2" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
+      <x:c r="I2" s="11"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -626,14 +639,14 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="7.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>标识</x:v>
       </x:c>
@@ -644,22 +657,20 @@
         <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>宽度</x:v>
+        <x:v>高X宽</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
-        <x:v>高度</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>能耗</x:v>
+        <x:v>贴图路径</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>贴图路径</x:v>
-      </x:c>
-      <x:c r="H1" s="10" t="str">
         <x:v>仓储容量</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="H1" s="10"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
         <x:v>function_radar</x:v>
       </x:c>
@@ -669,23 +680,21 @@
       <x:c r="C2" s="11" t="str">
         <x:v>基础功能模块。现阶段暂无额外参数。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
-        <x:v>1</x:v>
+      <x:c r="D2" s="11" t="str">
+        <x:v>1x1</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>res://data/assets/modules/function_radar.png</x:v>
       </x:c>
-      <x:c r="H2" s="11" t="n">
+      <x:c r="G2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3">
+      <x:c r="H2" s="11"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="11" t="str">
         <x:v>function_cargo_hold</x:v>
       </x:c>
@@ -695,21 +704,19 @@
       <x:c r="C3" s="11" t="str">
         <x:v>2×2 仓储模块，为当前 Run 提供 16 点模块仓储容量。</x:v>
       </x:c>
-      <x:c r="D3" s="11" t="n">
-        <x:v>2</x:v>
+      <x:c r="D3" s="11" t="str">
+        <x:v>2x2</x:v>
       </x:c>
       <x:c r="E3" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G3" s="11" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>res://data/assets/modules/function_cargo_hold.png</x:v>
       </x:c>
-      <x:c r="H3" s="11" t="n">
+      <x:c r="G3" s="11" t="n">
         <x:v>16</x:v>
       </x:c>
+      <x:c r="H3" s="11"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -723,13 +730,13 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="4.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>标识</x:v>
       </x:c>
@@ -740,19 +747,17 @@
         <x:v>描述</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>宽度</x:v>
+        <x:v>高X宽</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
-        <x:v>高度</x:v>
+        <x:v>能耗</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>能耗</x:v>
-      </x:c>
-      <x:c r="G1" s="10" t="str">
         <x:v>贴图路径</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="G1" s="10"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="11" t="str">
         <x:v>core_bridge</x:v>
       </x:c>
@@ -762,19 +767,18 @@
       <x:c r="C2" s="11" t="str">
         <x:v>飞船核心区域。核心模块被击毁时，飞船判定为沉没。</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
-        <x:v>2</x:v>
+      <x:c r="D2" s="11" t="str">
+        <x:v>2x2</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>res://data/assets/modules/core_bridge.png</x:v>
       </x:c>
-    </x:row>
+      <x:c r="G2" s="11"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>